<commit_message>
Mise à jour page SIGA
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lambris\prix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\siga\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F023C91-78E5-44C8-9C25-70C6BB20D3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D82F13-F1CA-411A-8C72-8F08F61C5D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
   <si>
     <t>path</t>
   </si>
@@ -59,64 +59,457 @@
     <t/>
   </si>
   <si>
-    <t>m²</t>
-  </si>
-  <si>
-    <t>13010108</t>
-  </si>
-  <si>
-    <t>13010109</t>
-  </si>
-  <si>
-    <t>13010110</t>
-  </si>
-  <si>
-    <t>13010111</t>
-  </si>
-  <si>
-    <t>13010112</t>
-  </si>
-  <si>
-    <t>Maestro MAF-002 millim</t>
-  </si>
-  <si>
-    <t>Maestro MAF-005 cristo</t>
-  </si>
-  <si>
-    <t>Maestro MAF-009 sarezzi</t>
-  </si>
-  <si>
-    <t>Maestro MAF-00080 blanc sat.</t>
-  </si>
-  <si>
-    <t>Maestro NOVO blanc brillant 0003</t>
-  </si>
-  <si>
-    <t>maf-005 cristo</t>
-  </si>
-  <si>
-    <t>maf-009 sarezzi</t>
-  </si>
-  <si>
-    <t>maf 00080</t>
-  </si>
-  <si>
-    <t>726158</t>
-  </si>
-  <si>
-    <t>galerie/millim.jpg</t>
-  </si>
-  <si>
-    <t>galerie/cristo.jpg</t>
-  </si>
-  <si>
-    <t>galerie/sarezzi.jpg</t>
-  </si>
-  <si>
-    <t>galerie/blanc-sat.jpg</t>
-  </si>
-  <si>
-    <t>galerie/blanc-brillant.jpg</t>
+    <t>59200000</t>
+  </si>
+  <si>
+    <t>59200002</t>
+  </si>
+  <si>
+    <t>59200004</t>
+  </si>
+  <si>
+    <t>59200006</t>
+  </si>
+  <si>
+    <t>59200008</t>
+  </si>
+  <si>
+    <t>59200010</t>
+  </si>
+  <si>
+    <t>59200016</t>
+  </si>
+  <si>
+    <t>59200018</t>
+  </si>
+  <si>
+    <t>59200020</t>
+  </si>
+  <si>
+    <t>59200024</t>
+  </si>
+  <si>
+    <t>59200026</t>
+  </si>
+  <si>
+    <t>59200030</t>
+  </si>
+  <si>
+    <t>59200034</t>
+  </si>
+  <si>
+    <t>59200036</t>
+  </si>
+  <si>
+    <t>59200038</t>
+  </si>
+  <si>
+    <t>59200040</t>
+  </si>
+  <si>
+    <t>59200042</t>
+  </si>
+  <si>
+    <t>59200050</t>
+  </si>
+  <si>
+    <t>59200051</t>
+  </si>
+  <si>
+    <t>59200052</t>
+  </si>
+  <si>
+    <t>59200054</t>
+  </si>
+  <si>
+    <t>59200055</t>
+  </si>
+  <si>
+    <t>59200056</t>
+  </si>
+  <si>
+    <t>59200057</t>
+  </si>
+  <si>
+    <t>59200058</t>
+  </si>
+  <si>
+    <t>592000585</t>
+  </si>
+  <si>
+    <t>592000586</t>
+  </si>
+  <si>
+    <t>59200060</t>
+  </si>
+  <si>
+    <t>59200061</t>
+  </si>
+  <si>
+    <t>59200062</t>
+  </si>
+  <si>
+    <t>59200063</t>
+  </si>
+  <si>
+    <t>59200070</t>
+  </si>
+  <si>
+    <t>59200072</t>
+  </si>
+  <si>
+    <t>59200073</t>
+  </si>
+  <si>
+    <t>59200074</t>
+  </si>
+  <si>
+    <t>59200075</t>
+  </si>
+  <si>
+    <t>59200076</t>
+  </si>
+  <si>
+    <t>59200080</t>
+  </si>
+  <si>
+    <t>Siga Twinet 20mmx50m</t>
+  </si>
+  <si>
+    <t>Siga Sicral 40mx60mm</t>
+  </si>
+  <si>
+    <t>Siga Sicral 40mx170mm</t>
+  </si>
+  <si>
+    <t>Siga Rissan 25mx60mm</t>
+  </si>
+  <si>
+    <t>Siga Rissan 25mx100mm</t>
+  </si>
+  <si>
+    <t>Siga Rissan 25mx150mm</t>
+  </si>
+  <si>
+    <t>Siga Primur 12x4mm -8m</t>
+  </si>
+  <si>
+    <t>Siga Primur boudin 600ml</t>
+  </si>
+  <si>
+    <t>Siga Primur 310ml</t>
+  </si>
+  <si>
+    <t>Siga Corvum 30/30 -25m</t>
+  </si>
+  <si>
+    <t>Siga Corvum 12/48mm -25m</t>
+  </si>
+  <si>
+    <t>Siga Docksin 1kg</t>
+  </si>
+  <si>
+    <t>Siga Wigluv 60  -60mmx40m</t>
+  </si>
+  <si>
+    <t>Siga Wigluv 60 20/40  -60mmx25m</t>
+  </si>
+  <si>
+    <t>Siga Wigluv 100  -100mmx25m</t>
+  </si>
+  <si>
+    <t>Siga Wigluv 150  -150mmx25m</t>
+  </si>
+  <si>
+    <t>Siga Wigluv black 60mmx40m</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 20  -25mx 50/85 (blanc troué)</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 20  -25mx 100mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 20  -25mx 150mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 20  -25mx 200mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS 20  -25mx 75mm (blanc)</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS 20  -25mx 100mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS 20  -25mx 150mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS 20  -25mx 200mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS 20  -25mx 250mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS 20  -25mx 300mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 2  -50/85</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 2  -25mx 100mm (troué)</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 2  -25mx 150mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim 2  -25mx 200mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS2 - 75mm 25m</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS2 - 100mm (noir plein)</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS2 - 150mm en 25m</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS2 - 200mm x20m</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS2 - 250mm</t>
+  </si>
+  <si>
+    <t>Siga Fentrim IS2 - 300mm</t>
+  </si>
+  <si>
+    <t>Siga Farmer 60mmx15m</t>
+  </si>
+  <si>
+    <t>6610-2050</t>
+  </si>
+  <si>
+    <t>4510-6040</t>
+  </si>
+  <si>
+    <t>4510-17040</t>
+  </si>
+  <si>
+    <t>2510-6025</t>
+  </si>
+  <si>
+    <t>2510-10025</t>
+  </si>
+  <si>
+    <t>2510-15025</t>
+  </si>
+  <si>
+    <t>3540-1208</t>
+  </si>
+  <si>
+    <t>3520</t>
+  </si>
+  <si>
+    <t>3510</t>
+  </si>
+  <si>
+    <t>5200-303025</t>
+  </si>
+  <si>
+    <t>5200-124825</t>
+  </si>
+  <si>
+    <t>5910</t>
+  </si>
+  <si>
+    <t>7510-6040</t>
+  </si>
+  <si>
+    <t>7510-6025</t>
+  </si>
+  <si>
+    <t>7510-10025</t>
+  </si>
+  <si>
+    <t>7510-15025</t>
+  </si>
+  <si>
+    <t>7509-6040</t>
+  </si>
+  <si>
+    <t>9511-508525</t>
+  </si>
+  <si>
+    <t>9511-158525</t>
+  </si>
+  <si>
+    <t>9511-1513525</t>
+  </si>
+  <si>
+    <t>9511-1518525</t>
+  </si>
+  <si>
+    <t>9611-156025</t>
+  </si>
+  <si>
+    <t>9611-158525</t>
+  </si>
+  <si>
+    <t>9611-1513525</t>
+  </si>
+  <si>
+    <t>9611-1518525</t>
+  </si>
+  <si>
+    <t>9611-1523525</t>
+  </si>
+  <si>
+    <t>9611-</t>
+  </si>
+  <si>
+    <t>9512-508525</t>
+  </si>
+  <si>
+    <t>9512-158525</t>
+  </si>
+  <si>
+    <t>9512-1513525</t>
+  </si>
+  <si>
+    <t>9512-1518525</t>
+  </si>
+  <si>
+    <t>9612-156025</t>
+  </si>
+  <si>
+    <t>9612-158525</t>
+  </si>
+  <si>
+    <t>9612-1513525</t>
+  </si>
+  <si>
+    <t>9612-1518525</t>
+  </si>
+  <si>
+    <t>9612-1523525</t>
+  </si>
+  <si>
+    <t>6500-6015</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Twinet_20_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Sicrall_60_B.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Sicrall_170_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Rissan_60_B.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Rissan_100_B.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Rissan_150mm_packshot_B_2510-15025.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Corvum_30-30_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Corvum_12-48_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Wigluv_60_500x500.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Wigluv_100_500x500.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Wigluv_150_500x500.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Wigluv_black_60mm_packshot_A_7509-6040.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Fentrim_20_50-85_packshot_A_9511-508525.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Fentrim_20_100mm_packshot_A_9511-158525.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_20_150mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_20_200mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_20_100mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_20_200mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_20_250mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_20_300mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_2_50-85_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_2_100mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_2_150mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_2_200mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_2_75mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_2_100mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_2_150mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_2_200mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_2_250mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Fentrim_IS_2_300mm_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Fentrim_IS_20_75mm_packshot_A_9611-156025.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Fentrim_IS_20_150mm_packshot_A_9611-1513525.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Wigluv_2040_500x500.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Primur_cartridge_B.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Primur_Rolle_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/Primur_tubular_bag_A.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/SIGA_Dockskin_1kg_packshot_A_5930.png</t>
+  </si>
+  <si>
+    <t>/siga/galerie/siga-farmer.png</t>
   </si>
 </sst>
 </file>
@@ -188,7 +581,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -227,19 +620,10 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -259,6 +643,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -597,12 +984,12 @@
   <dimension ref="A1:G450"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="58.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="64.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.88671875" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" style="16" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.77734375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -622,668 +1009,1059 @@
       <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="14" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="19">
+        <v>39.020000000000003</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="20">
+        <v>10</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="19">
+        <v>32.78</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="20">
+        <v>3</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="19">
+        <v>120.37</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="20">
+        <v>2</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="19">
+        <v>25.43</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="20">
+        <v>19</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="19">
+        <v>56.410000000000004</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="20">
+        <v>9</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="19">
+        <v>80.95</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="20">
+        <v>3</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="19">
+        <v>20.67</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="20">
+        <v>10</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="19">
+        <v>17.18</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="20">
+        <v>12</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="19">
+        <v>10.99</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="20">
+        <v>13</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="19">
+        <v>48.07</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="20">
+        <v>7</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="19">
+        <v>48.07</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="20">
+        <v>10</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="19">
+        <v>30.44</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="20">
+        <v>4</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="19">
+        <v>43.37</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="20">
+        <v>14</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="19">
+        <v>45.35</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="20">
+        <v>3</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="19">
+        <v>59.58</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="20">
+        <v>6</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="19">
+        <v>83.76</v>
+      </c>
+      <c r="E17" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="F17" s="20">
         <v>13</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="G17" s="21" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="19">
+        <v>63.68</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="20">
+        <v>0</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="19">
+        <v>95.93</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" s="20">
+        <v>10</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="19">
+        <v>66.540000000000006</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="20">
+        <v>10</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="19">
+        <v>99.89</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" s="20">
+        <v>54</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="19">
+        <v>138.11000000000001</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" s="20">
+        <v>0</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="19">
+        <v>55.95</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="20">
         <v>7</v>
       </c>
-      <c r="D2" s="22">
-        <v>15</v>
-      </c>
-      <c r="E2" s="20" t="s">
+      <c r="G23" s="21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="19">
+        <v>66.540000000000006</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" s="20">
+        <v>12</v>
+      </c>
+      <c r="G24" s="21" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" s="19">
+        <v>99.89</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="F25" s="20">
+        <v>28</v>
+      </c>
+      <c r="G25" s="21" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="19">
+        <v>138.11000000000001</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F26" s="20">
         <v>8</v>
       </c>
-      <c r="F2" s="23">
-        <v>91.021000000006609</v>
-      </c>
-      <c r="G2" s="24" t="s">
+      <c r="G26" s="21" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="19">
+        <v>169.1</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" s="20">
+        <v>1</v>
+      </c>
+      <c r="G27" s="21" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28" s="19">
+        <v>198.63</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F28" s="20">
+        <v>0</v>
+      </c>
+      <c r="G28" s="21" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="19">
+        <v>99.62</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F29" s="20">
+        <v>10</v>
+      </c>
+      <c r="G29" s="21" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="19">
+        <v>70.05</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F30" s="20">
+        <v>13</v>
+      </c>
+      <c r="G30" s="21" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" s="19">
+        <v>104.97</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F31" s="20">
+        <v>20</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="19">
+        <v>143.91</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" s="20">
+        <v>12</v>
+      </c>
+      <c r="G32" s="21" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="19">
+        <v>58.93</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F33" s="20">
+        <v>3</v>
+      </c>
+      <c r="G33" s="21" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D34" s="19">
+        <v>70.05</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="F34" s="20">
+        <v>0</v>
+      </c>
+      <c r="G34" s="21" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="D35" s="19">
+        <v>104.97</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" s="20">
+        <v>16</v>
+      </c>
+      <c r="G35" s="21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="19">
+        <v>143.91</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="F36" s="20">
+        <v>0</v>
+      </c>
+      <c r="G36" s="21" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" s="19">
+        <v>174.41</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F37" s="20">
+        <v>0</v>
+      </c>
+      <c r="G37" s="21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="D38" s="19">
+        <v>189.69</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F38" s="20">
+        <v>0</v>
+      </c>
+      <c r="G38" s="21" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="22">
-        <v>15</v>
-      </c>
-      <c r="E3" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="23">
-        <v>125.46600000000014</v>
-      </c>
-      <c r="G3" s="24" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="22">
-        <v>15</v>
-      </c>
-      <c r="E4" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="23">
-        <v>78.721999999996953</v>
-      </c>
-      <c r="G4" s="24" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="22">
-        <v>15</v>
-      </c>
-      <c r="E5" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="23">
-        <v>84.876000000000431</v>
-      </c>
-      <c r="G5" s="24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="21" t="s">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="D39" s="19">
+        <v>27.42</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F39" s="20">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="22">
-        <v>26.18</v>
-      </c>
-      <c r="E6" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="23">
-        <v>93.057999999999993</v>
-      </c>
-      <c r="G6" s="24" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="8"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="8"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="8"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="8"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="8"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="8"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="8"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="8"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="8"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="8"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="15"/>
-      <c r="B12" s="9"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="8"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="9"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="9"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="8"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="8"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="15"/>
-      <c r="B15" s="9"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="9"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="9"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="8"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="15"/>
-      <c r="B17" s="9"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="9"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="15"/>
-      <c r="B18" s="9"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="9"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="9"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="8"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="9"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="8"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="9"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="8"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="9"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="8"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="9"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="8"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="5"/>
-      <c r="B24" s="9"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="8"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
-      <c r="B25" s="8"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="8"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="15"/>
-      <c r="B26" s="9"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="9"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="5"/>
-      <c r="B27" s="9"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="8"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
-      <c r="B28" s="8"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="8"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="8"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="5"/>
-      <c r="B30" s="8"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="8"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="5"/>
-      <c r="B31" s="8"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="17"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="5"/>
-      <c r="B32" s="8"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="17"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="5"/>
-      <c r="B33" s="8"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="17"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="5"/>
-      <c r="B34" s="8"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="17"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="5"/>
-      <c r="B35" s="8"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="17"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="5"/>
-      <c r="B36" s="8"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="17"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="5"/>
-      <c r="B37" s="8"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="17"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="5"/>
-      <c r="B38" s="8"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="17"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="5"/>
-      <c r="B39" s="8"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="17"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" s="21" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="5"/>
-      <c r="B40" s="8"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="17"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B40" s="18"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="21"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="5"/>
       <c r="B41" s="8"/>
       <c r="D41" s="12"/>
       <c r="E41" s="8"/>
-      <c r="F41" s="17"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F41" s="15"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="5"/>
       <c r="B42" s="8"/>
       <c r="D42" s="12"/>
       <c r="E42" s="8"/>
-      <c r="F42" s="17"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F42" s="15"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="5"/>
       <c r="B43" s="8"/>
       <c r="D43" s="12"/>
       <c r="E43" s="8"/>
-      <c r="F43" s="17"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F43" s="15"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="5"/>
       <c r="B44" s="8"/>
       <c r="D44" s="12"/>
       <c r="E44" s="8"/>
-      <c r="F44" s="17"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F44" s="15"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="5"/>
       <c r="B45" s="8"/>
       <c r="D45" s="12"/>
       <c r="E45" s="8"/>
-      <c r="F45" s="17"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F45" s="15"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="5"/>
       <c r="B46" s="8"/>
       <c r="D46" s="12"/>
       <c r="E46" s="8"/>
-      <c r="F46" s="17"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F46" s="15"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="5"/>
       <c r="B47" s="8"/>
       <c r="D47" s="12"/>
       <c r="E47" s="8"/>
-      <c r="F47" s="17"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F47" s="15"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="5"/>
       <c r="B48" s="8"/>
       <c r="D48" s="12"/>
       <c r="E48" s="8"/>
-      <c r="F48" s="17"/>
+      <c r="F48" s="15"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="5"/>
       <c r="B49" s="8"/>
       <c r="D49" s="12"/>
       <c r="E49" s="8"/>
-      <c r="F49" s="17"/>
+      <c r="F49" s="15"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="5"/>
       <c r="B50" s="8"/>
       <c r="D50" s="12"/>
       <c r="E50" s="8"/>
-      <c r="F50" s="17"/>
+      <c r="F50" s="15"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="5"/>
       <c r="B51" s="8"/>
       <c r="D51" s="12"/>
       <c r="E51" s="8"/>
-      <c r="F51" s="17"/>
+      <c r="F51" s="15"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="5"/>
       <c r="B52" s="8"/>
       <c r="D52" s="12"/>
       <c r="E52" s="8"/>
-      <c r="F52" s="17"/>
+      <c r="F52" s="15"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="5"/>
       <c r="B53" s="8"/>
       <c r="D53" s="12"/>
       <c r="E53" s="8"/>
-      <c r="F53" s="17"/>
+      <c r="F53" s="15"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="5"/>
       <c r="B54" s="8"/>
       <c r="D54" s="12"/>
       <c r="E54" s="8"/>
-      <c r="F54" s="17"/>
+      <c r="F54" s="15"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="5"/>
       <c r="B55" s="8"/>
       <c r="D55" s="12"/>
       <c r="E55" s="8"/>
-      <c r="F55" s="17"/>
+      <c r="F55" s="15"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="5"/>
       <c r="B56" s="8"/>
       <c r="D56" s="12"/>
       <c r="E56" s="8"/>
-      <c r="F56" s="17"/>
+      <c r="F56" s="15"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="5"/>
       <c r="B57" s="8"/>
       <c r="D57" s="12"/>
       <c r="E57" s="8"/>
-      <c r="F57" s="17"/>
+      <c r="F57" s="15"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="5"/>
       <c r="B58" s="8"/>
       <c r="D58" s="12"/>
       <c r="E58" s="8"/>
-      <c r="F58" s="17"/>
+      <c r="F58" s="15"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
       <c r="B59" s="8"/>
       <c r="D59" s="12"/>
       <c r="E59" s="8"/>
-      <c r="F59" s="17"/>
+      <c r="F59" s="15"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="5"/>
       <c r="B60" s="8"/>
       <c r="D60" s="12"/>
       <c r="E60" s="8"/>
-      <c r="F60" s="17"/>
+      <c r="F60" s="15"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="5"/>
       <c r="B61" s="8"/>
       <c r="D61" s="12"/>
       <c r="E61" s="8"/>
-      <c r="F61" s="17"/>
+      <c r="F61" s="15"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="5"/>
       <c r="B62" s="8"/>
       <c r="D62" s="12"/>
       <c r="E62" s="8"/>
-      <c r="F62" s="17"/>
+      <c r="F62" s="15"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="5"/>
       <c r="B63" s="8"/>
       <c r="D63" s="12"/>
       <c r="E63" s="8"/>
-      <c r="F63" s="17"/>
+      <c r="F63" s="15"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="5"/>
       <c r="B64" s="8"/>
       <c r="D64" s="12"/>
       <c r="E64" s="8"/>
-      <c r="F64" s="17"/>
+      <c r="F64" s="15"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="5"/>
       <c r="B65" s="8"/>
       <c r="D65" s="12"/>
       <c r="E65" s="8"/>
-      <c r="F65" s="17"/>
+      <c r="F65" s="15"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="5"/>
       <c r="B66" s="8"/>
       <c r="D66" s="12"/>
       <c r="E66" s="8"/>
-      <c r="F66" s="17"/>
+      <c r="F66" s="15"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="5"/>
       <c r="B67" s="8"/>
       <c r="D67" s="12"/>
       <c r="E67" s="8"/>
-      <c r="F67" s="17"/>
+      <c r="F67" s="15"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="5"/>
       <c r="B68" s="8"/>
       <c r="D68" s="12"/>
       <c r="E68" s="8"/>
-      <c r="F68" s="17"/>
+      <c r="F68" s="15"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="5"/>
       <c r="B69" s="8"/>
       <c r="D69" s="12"/>
       <c r="E69" s="8"/>
-      <c r="F69" s="17"/>
+      <c r="F69" s="15"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="5"/>
       <c r="B70" s="8"/>
       <c r="D70" s="12"/>
       <c r="E70" s="8"/>
-      <c r="F70" s="17"/>
+      <c r="F70" s="15"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="5"/>
       <c r="B71" s="8"/>
       <c r="D71" s="12"/>
       <c r="E71" s="8"/>
-      <c r="F71" s="17"/>
+      <c r="F71" s="15"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="5"/>
       <c r="B72" s="8"/>
       <c r="D72" s="12"/>
       <c r="E72" s="8"/>
-      <c r="F72" s="17"/>
+      <c r="F72" s="15"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="5"/>
       <c r="B73" s="8"/>
       <c r="D73" s="12"/>
       <c r="E73" s="8"/>
-      <c r="F73" s="17"/>
+      <c r="F73" s="15"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="5"/>
       <c r="B74" s="8"/>
       <c r="D74" s="12"/>
       <c r="E74" s="8"/>
-      <c r="F74" s="17"/>
+      <c r="F74" s="15"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="5"/>
       <c r="B75" s="8"/>
       <c r="D75" s="12"/>
       <c r="E75" s="8"/>
-      <c r="F75" s="17"/>
+      <c r="F75" s="15"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="5"/>
       <c r="B76" s="8"/>
       <c r="D76" s="12"/>
       <c r="E76" s="8"/>
-      <c r="F76" s="17"/>
+      <c r="F76" s="15"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="5"/>
       <c r="B77" s="8"/>
       <c r="D77" s="12"/>
       <c r="E77" s="8"/>
-      <c r="F77" s="17"/>
+      <c r="F77" s="15"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="5"/>
       <c r="B78" s="8"/>
       <c r="D78" s="12"/>
       <c r="E78" s="8"/>
-      <c r="F78" s="17"/>
+      <c r="F78" s="15"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="5"/>
       <c r="B79" s="8"/>
       <c r="D79" s="12"/>
       <c r="E79" s="8"/>
-      <c r="F79" s="17"/>
+      <c r="F79" s="15"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="5"/>
       <c r="B80" s="8"/>
       <c r="D80" s="12"/>
       <c r="E80" s="8"/>
-      <c r="F80" s="17"/>
+      <c r="F80" s="15"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="5"/>
@@ -1291,7 +2069,7 @@
       <c r="C81" s="4"/>
       <c r="D81" s="12"/>
       <c r="E81" s="8"/>
-      <c r="F81" s="17"/>
+      <c r="F81" s="15"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="5"/>
@@ -1299,7 +2077,7 @@
       <c r="C82" s="4"/>
       <c r="D82" s="12"/>
       <c r="E82" s="8"/>
-      <c r="F82" s="17"/>
+      <c r="F82" s="15"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="5"/>
@@ -1307,7 +2085,7 @@
       <c r="C83" s="4"/>
       <c r="D83" s="12"/>
       <c r="E83" s="8"/>
-      <c r="F83" s="17"/>
+      <c r="F83" s="15"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="5"/>
@@ -1315,7 +2093,7 @@
       <c r="C84" s="4"/>
       <c r="D84" s="12"/>
       <c r="E84" s="8"/>
-      <c r="F84" s="17"/>
+      <c r="F84" s="15"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="5"/>
@@ -1323,7 +2101,7 @@
       <c r="C85" s="4"/>
       <c r="D85" s="12"/>
       <c r="E85" s="8"/>
-      <c r="F85" s="17"/>
+      <c r="F85" s="15"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="5"/>
@@ -1331,7 +2109,7 @@
       <c r="C86" s="4"/>
       <c r="D86" s="12"/>
       <c r="E86" s="8"/>
-      <c r="F86" s="17"/>
+      <c r="F86" s="15"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="5"/>
@@ -1339,7 +2117,7 @@
       <c r="C87" s="4"/>
       <c r="D87" s="12"/>
       <c r="E87" s="8"/>
-      <c r="F87" s="17"/>
+      <c r="F87" s="15"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="5"/>
@@ -1347,7 +2125,7 @@
       <c r="C88" s="4"/>
       <c r="D88" s="12"/>
       <c r="E88" s="8"/>
-      <c r="F88" s="17"/>
+      <c r="F88" s="15"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="5"/>
@@ -1355,7 +2133,7 @@
       <c r="C89" s="4"/>
       <c r="D89" s="12"/>
       <c r="E89" s="8"/>
-      <c r="F89" s="17"/>
+      <c r="F89" s="15"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="5"/>
@@ -1363,7 +2141,7 @@
       <c r="C90" s="4"/>
       <c r="D90" s="12"/>
       <c r="E90" s="8"/>
-      <c r="F90" s="17"/>
+      <c r="F90" s="15"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="5"/>
@@ -1371,7 +2149,7 @@
       <c r="C91" s="4"/>
       <c r="D91" s="12"/>
       <c r="E91" s="8"/>
-      <c r="F91" s="17"/>
+      <c r="F91" s="15"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="5"/>
@@ -1379,7 +2157,7 @@
       <c r="C92" s="4"/>
       <c r="D92" s="12"/>
       <c r="E92" s="8"/>
-      <c r="F92" s="17"/>
+      <c r="F92" s="15"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="5"/>
@@ -1387,7 +2165,7 @@
       <c r="C93" s="4"/>
       <c r="D93" s="12"/>
       <c r="E93" s="8"/>
-      <c r="F93" s="17"/>
+      <c r="F93" s="15"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="5"/>
@@ -1395,7 +2173,7 @@
       <c r="C94" s="4"/>
       <c r="D94" s="12"/>
       <c r="E94" s="8"/>
-      <c r="F94" s="17"/>
+      <c r="F94" s="15"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="5"/>
@@ -1403,7 +2181,7 @@
       <c r="C95" s="4"/>
       <c r="D95" s="12"/>
       <c r="E95" s="8"/>
-      <c r="F95" s="17"/>
+      <c r="F95" s="15"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="5"/>
@@ -1411,7 +2189,7 @@
       <c r="C96" s="4"/>
       <c r="D96" s="12"/>
       <c r="E96" s="8"/>
-      <c r="F96" s="17"/>
+      <c r="F96" s="15"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="5"/>
@@ -1419,7 +2197,7 @@
       <c r="C97" s="4"/>
       <c r="D97" s="12"/>
       <c r="E97" s="8"/>
-      <c r="F97" s="17"/>
+      <c r="F97" s="15"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="5"/>
@@ -1427,7 +2205,7 @@
       <c r="C98" s="4"/>
       <c r="D98" s="12"/>
       <c r="E98" s="8"/>
-      <c r="F98" s="17"/>
+      <c r="F98" s="15"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="5"/>
@@ -1435,7 +2213,7 @@
       <c r="C99" s="4"/>
       <c r="D99" s="12"/>
       <c r="E99" s="8"/>
-      <c r="F99" s="17"/>
+      <c r="F99" s="15"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="5"/>
@@ -1443,7 +2221,7 @@
       <c r="C100" s="4"/>
       <c r="D100" s="12"/>
       <c r="E100" s="8"/>
-      <c r="F100" s="17"/>
+      <c r="F100" s="15"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="5"/>
@@ -1451,7 +2229,7 @@
       <c r="C101" s="4"/>
       <c r="D101" s="12"/>
       <c r="E101" s="8"/>
-      <c r="F101" s="17"/>
+      <c r="F101" s="15"/>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="5"/>
@@ -1459,7 +2237,7 @@
       <c r="C102" s="4"/>
       <c r="D102" s="12"/>
       <c r="E102" s="8"/>
-      <c r="F102" s="17"/>
+      <c r="F102" s="15"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="5"/>
@@ -1467,7 +2245,7 @@
       <c r="C103" s="4"/>
       <c r="D103" s="12"/>
       <c r="E103" s="8"/>
-      <c r="F103" s="17"/>
+      <c r="F103" s="15"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="5"/>
@@ -1475,7 +2253,7 @@
       <c r="C104" s="4"/>
       <c r="D104" s="12"/>
       <c r="E104" s="8"/>
-      <c r="F104" s="17"/>
+      <c r="F104" s="15"/>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="5"/>
@@ -1483,7 +2261,7 @@
       <c r="C105" s="4"/>
       <c r="D105" s="12"/>
       <c r="E105" s="8"/>
-      <c r="F105" s="17"/>
+      <c r="F105" s="15"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="5"/>
@@ -1491,7 +2269,7 @@
       <c r="C106" s="4"/>
       <c r="D106" s="12"/>
       <c r="E106" s="8"/>
-      <c r="F106" s="17"/>
+      <c r="F106" s="15"/>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="5"/>
@@ -1499,7 +2277,7 @@
       <c r="C107" s="4"/>
       <c r="D107" s="12"/>
       <c r="E107" s="8"/>
-      <c r="F107" s="17"/>
+      <c r="F107" s="15"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="5"/>
@@ -1507,7 +2285,7 @@
       <c r="C108" s="4"/>
       <c r="D108" s="12"/>
       <c r="E108" s="8"/>
-      <c r="F108" s="17"/>
+      <c r="F108" s="15"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="5"/>
@@ -1515,7 +2293,7 @@
       <c r="C109" s="4"/>
       <c r="D109" s="12"/>
       <c r="E109" s="8"/>
-      <c r="F109" s="17"/>
+      <c r="F109" s="15"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="5"/>
@@ -1523,7 +2301,7 @@
       <c r="C110" s="4"/>
       <c r="D110" s="12"/>
       <c r="E110" s="8"/>
-      <c r="F110" s="17"/>
+      <c r="F110" s="15"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="5"/>
@@ -1531,7 +2309,7 @@
       <c r="C111" s="4"/>
       <c r="D111" s="12"/>
       <c r="E111" s="8"/>
-      <c r="F111" s="17"/>
+      <c r="F111" s="15"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="5"/>
@@ -1539,7 +2317,7 @@
       <c r="C112" s="4"/>
       <c r="D112" s="12"/>
       <c r="E112" s="8"/>
-      <c r="F112" s="17"/>
+      <c r="F112" s="15"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="5"/>
@@ -1547,7 +2325,7 @@
       <c r="C113" s="4"/>
       <c r="D113" s="12"/>
       <c r="E113" s="8"/>
-      <c r="F113" s="17"/>
+      <c r="F113" s="15"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="5"/>
@@ -1555,7 +2333,7 @@
       <c r="C114" s="4"/>
       <c r="D114" s="12"/>
       <c r="E114" s="8"/>
-      <c r="F114" s="17"/>
+      <c r="F114" s="15"/>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="5"/>
@@ -1563,7 +2341,7 @@
       <c r="C115" s="4"/>
       <c r="D115" s="12"/>
       <c r="E115" s="8"/>
-      <c r="F115" s="17"/>
+      <c r="F115" s="15"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="5"/>
@@ -1571,1176 +2349,1176 @@
       <c r="C116" s="4"/>
       <c r="D116" s="12"/>
       <c r="E116" s="8"/>
-      <c r="F116" s="17"/>
+      <c r="F116" s="15"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="5"/>
       <c r="B117" s="8"/>
       <c r="D117" s="12"/>
       <c r="E117" s="8"/>
-      <c r="F117" s="17"/>
+      <c r="F117" s="15"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="5"/>
       <c r="B118" s="8"/>
       <c r="D118" s="12"/>
       <c r="E118" s="8"/>
-      <c r="F118" s="17"/>
+      <c r="F118" s="15"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="5"/>
       <c r="B119" s="8"/>
       <c r="D119" s="12"/>
       <c r="E119" s="8"/>
-      <c r="F119" s="17"/>
+      <c r="F119" s="15"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="5"/>
       <c r="B120" s="8"/>
       <c r="D120" s="12"/>
       <c r="E120" s="8"/>
-      <c r="F120" s="17"/>
+      <c r="F120" s="15"/>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="5"/>
       <c r="B121" s="8"/>
       <c r="D121" s="12"/>
       <c r="E121" s="8"/>
-      <c r="F121" s="17"/>
+      <c r="F121" s="15"/>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="5"/>
       <c r="B122" s="8"/>
       <c r="D122" s="12"/>
       <c r="E122" s="8"/>
-      <c r="F122" s="17"/>
+      <c r="F122" s="15"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="5"/>
       <c r="B123" s="8"/>
       <c r="D123" s="12"/>
       <c r="E123" s="8"/>
-      <c r="F123" s="17"/>
+      <c r="F123" s="15"/>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="5"/>
       <c r="B124" s="8"/>
       <c r="D124" s="12"/>
       <c r="E124" s="8"/>
-      <c r="F124" s="17"/>
+      <c r="F124" s="15"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="5"/>
       <c r="B125" s="8"/>
       <c r="D125" s="12"/>
       <c r="E125" s="8"/>
-      <c r="F125" s="17"/>
+      <c r="F125" s="15"/>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="5"/>
       <c r="B126" s="8"/>
       <c r="D126" s="12"/>
       <c r="E126" s="8"/>
-      <c r="F126" s="17"/>
+      <c r="F126" s="15"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="5"/>
       <c r="B127" s="8"/>
       <c r="D127" s="12"/>
       <c r="E127" s="8"/>
-      <c r="F127" s="17"/>
+      <c r="F127" s="15"/>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="5"/>
       <c r="B128" s="8"/>
       <c r="D128" s="12"/>
       <c r="E128" s="8"/>
-      <c r="F128" s="17"/>
+      <c r="F128" s="15"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="5"/>
       <c r="B129" s="8"/>
       <c r="D129" s="12"/>
       <c r="E129" s="8"/>
-      <c r="F129" s="17"/>
+      <c r="F129" s="15"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="5"/>
       <c r="B130" s="8"/>
       <c r="D130" s="12"/>
       <c r="E130" s="8"/>
-      <c r="F130" s="17"/>
+      <c r="F130" s="15"/>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="5"/>
       <c r="B131" s="8"/>
       <c r="D131" s="12"/>
       <c r="E131" s="8"/>
-      <c r="F131" s="17"/>
+      <c r="F131" s="15"/>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="5"/>
       <c r="B132" s="8"/>
       <c r="D132" s="12"/>
       <c r="E132" s="8"/>
-      <c r="F132" s="17"/>
+      <c r="F132" s="15"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="5"/>
       <c r="B133" s="8"/>
       <c r="D133" s="12"/>
       <c r="E133" s="8"/>
-      <c r="F133" s="17"/>
+      <c r="F133" s="15"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="5"/>
       <c r="B134" s="8"/>
       <c r="D134" s="12"/>
       <c r="E134" s="8"/>
-      <c r="F134" s="17"/>
+      <c r="F134" s="15"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="5"/>
       <c r="B135" s="8"/>
       <c r="D135" s="12"/>
       <c r="E135" s="8"/>
-      <c r="F135" s="17"/>
+      <c r="F135" s="15"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="5"/>
       <c r="B136" s="8"/>
       <c r="D136" s="12"/>
       <c r="E136" s="8"/>
-      <c r="F136" s="17"/>
+      <c r="F136" s="15"/>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="5"/>
       <c r="B137" s="8"/>
       <c r="D137" s="12"/>
       <c r="E137" s="8"/>
-      <c r="F137" s="17"/>
+      <c r="F137" s="15"/>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="5"/>
       <c r="B138" s="8"/>
       <c r="D138" s="12"/>
       <c r="E138" s="8"/>
-      <c r="F138" s="17"/>
+      <c r="F138" s="15"/>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="5"/>
       <c r="B139" s="8"/>
       <c r="D139" s="12"/>
       <c r="E139" s="8"/>
-      <c r="F139" s="17"/>
+      <c r="F139" s="15"/>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="5"/>
       <c r="B140" s="8"/>
       <c r="D140" s="12"/>
       <c r="E140" s="8"/>
-      <c r="F140" s="17"/>
+      <c r="F140" s="15"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="5"/>
       <c r="B141" s="8"/>
       <c r="D141" s="12"/>
       <c r="E141" s="8"/>
-      <c r="F141" s="17"/>
+      <c r="F141" s="15"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="5"/>
       <c r="B142" s="8"/>
       <c r="D142" s="12"/>
       <c r="E142" s="8"/>
-      <c r="F142" s="17"/>
+      <c r="F142" s="15"/>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="5"/>
       <c r="B143" s="8"/>
       <c r="D143" s="12"/>
       <c r="E143" s="8"/>
-      <c r="F143" s="17"/>
+      <c r="F143" s="15"/>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="5"/>
       <c r="B144" s="8"/>
       <c r="D144" s="12"/>
       <c r="E144" s="8"/>
-      <c r="F144" s="17"/>
+      <c r="F144" s="15"/>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="5"/>
       <c r="B145" s="8"/>
       <c r="D145" s="12"/>
       <c r="E145" s="8"/>
-      <c r="F145" s="17"/>
+      <c r="F145" s="15"/>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="5"/>
       <c r="B146" s="8"/>
       <c r="D146" s="12"/>
       <c r="E146" s="8"/>
-      <c r="F146" s="17"/>
+      <c r="F146" s="15"/>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="5"/>
       <c r="B147" s="8"/>
       <c r="D147" s="12"/>
       <c r="E147" s="8"/>
-      <c r="F147" s="17"/>
+      <c r="F147" s="15"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="5"/>
       <c r="B148" s="8"/>
       <c r="D148" s="12"/>
       <c r="E148" s="8"/>
-      <c r="F148" s="17"/>
+      <c r="F148" s="15"/>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="5"/>
       <c r="B149" s="8"/>
       <c r="D149" s="12"/>
       <c r="E149" s="8"/>
-      <c r="F149" s="17"/>
+      <c r="F149" s="15"/>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="5"/>
       <c r="B150" s="8"/>
       <c r="D150" s="12"/>
       <c r="E150" s="8"/>
-      <c r="F150" s="17"/>
+      <c r="F150" s="15"/>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="5"/>
       <c r="B151" s="8"/>
       <c r="D151" s="12"/>
       <c r="E151" s="8"/>
-      <c r="F151" s="17"/>
+      <c r="F151" s="15"/>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="5"/>
       <c r="B152" s="8"/>
       <c r="D152" s="12"/>
       <c r="E152" s="8"/>
-      <c r="F152" s="17"/>
+      <c r="F152" s="15"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="5"/>
       <c r="B153" s="8"/>
       <c r="D153" s="12"/>
       <c r="E153" s="8"/>
-      <c r="F153" s="17"/>
+      <c r="F153" s="15"/>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="5"/>
       <c r="B154" s="8"/>
       <c r="D154" s="12"/>
       <c r="E154" s="8"/>
-      <c r="F154" s="17"/>
+      <c r="F154" s="15"/>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="5"/>
       <c r="B155" s="8"/>
       <c r="D155" s="12"/>
       <c r="E155" s="8"/>
-      <c r="F155" s="17"/>
+      <c r="F155" s="15"/>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="5"/>
       <c r="B156" s="8"/>
       <c r="D156" s="12"/>
       <c r="E156" s="8"/>
-      <c r="F156" s="17"/>
+      <c r="F156" s="15"/>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="5"/>
       <c r="B157" s="8"/>
       <c r="D157" s="12"/>
       <c r="E157" s="8"/>
-      <c r="F157" s="17"/>
+      <c r="F157" s="15"/>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="5"/>
       <c r="B158" s="8"/>
       <c r="D158" s="12"/>
       <c r="E158" s="8"/>
-      <c r="F158" s="17"/>
+      <c r="F158" s="15"/>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="5"/>
       <c r="B159" s="8"/>
       <c r="D159" s="12"/>
       <c r="E159" s="8"/>
-      <c r="F159" s="17"/>
+      <c r="F159" s="15"/>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="5"/>
       <c r="B160" s="8"/>
       <c r="D160" s="12"/>
       <c r="E160" s="8"/>
-      <c r="F160" s="17"/>
+      <c r="F160" s="15"/>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="5"/>
       <c r="B161" s="8"/>
       <c r="D161" s="12"/>
       <c r="E161" s="8"/>
-      <c r="F161" s="17"/>
+      <c r="F161" s="15"/>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="5"/>
       <c r="B162" s="8"/>
       <c r="D162" s="12"/>
       <c r="E162" s="8"/>
-      <c r="F162" s="17"/>
+      <c r="F162" s="15"/>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="5"/>
       <c r="B163" s="8"/>
       <c r="D163" s="12"/>
       <c r="E163" s="8"/>
-      <c r="F163" s="17"/>
+      <c r="F163" s="15"/>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="5"/>
       <c r="B164" s="8"/>
       <c r="D164" s="12"/>
       <c r="E164" s="8"/>
-      <c r="F164" s="17"/>
+      <c r="F164" s="15"/>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="5"/>
       <c r="B165" s="8"/>
       <c r="D165" s="12"/>
       <c r="E165" s="8"/>
-      <c r="F165" s="17"/>
+      <c r="F165" s="15"/>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="5"/>
       <c r="B166" s="8"/>
       <c r="D166" s="12"/>
       <c r="E166" s="8"/>
-      <c r="F166" s="17"/>
+      <c r="F166" s="15"/>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" s="5"/>
       <c r="B167" s="8"/>
       <c r="D167" s="12"/>
       <c r="E167" s="8"/>
-      <c r="F167" s="17"/>
+      <c r="F167" s="15"/>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="5"/>
       <c r="B168" s="8"/>
       <c r="D168" s="12"/>
       <c r="E168" s="8"/>
-      <c r="F168" s="17"/>
+      <c r="F168" s="15"/>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" s="5"/>
       <c r="B169" s="8"/>
       <c r="D169" s="12"/>
       <c r="E169" s="8"/>
-      <c r="F169" s="17"/>
+      <c r="F169" s="15"/>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" s="5"/>
       <c r="B170" s="8"/>
       <c r="D170" s="12"/>
       <c r="E170" s="8"/>
-      <c r="F170" s="17"/>
+      <c r="F170" s="15"/>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="5"/>
       <c r="B171" s="8"/>
       <c r="D171" s="12"/>
       <c r="E171" s="8"/>
-      <c r="F171" s="17"/>
+      <c r="F171" s="15"/>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" s="5"/>
       <c r="B172" s="8"/>
       <c r="D172" s="12"/>
       <c r="E172" s="8"/>
-      <c r="F172" s="17"/>
+      <c r="F172" s="15"/>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" s="5"/>
       <c r="B173" s="8"/>
       <c r="D173" s="12"/>
       <c r="E173" s="8"/>
-      <c r="F173" s="17"/>
+      <c r="F173" s="15"/>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" s="5"/>
       <c r="B174" s="8"/>
       <c r="D174" s="12"/>
       <c r="E174" s="8"/>
-      <c r="F174" s="17"/>
+      <c r="F174" s="15"/>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" s="5"/>
       <c r="B175" s="8"/>
       <c r="D175" s="12"/>
       <c r="E175" s="8"/>
-      <c r="F175" s="17"/>
+      <c r="F175" s="15"/>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" s="5"/>
       <c r="B176" s="8"/>
       <c r="D176" s="12"/>
       <c r="E176" s="8"/>
-      <c r="F176" s="17"/>
+      <c r="F176" s="15"/>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" s="5"/>
       <c r="B177" s="8"/>
       <c r="D177" s="12"/>
       <c r="E177" s="8"/>
-      <c r="F177" s="17"/>
+      <c r="F177" s="15"/>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" s="5"/>
       <c r="B178" s="8"/>
       <c r="D178" s="12"/>
       <c r="E178" s="8"/>
-      <c r="F178" s="17"/>
+      <c r="F178" s="15"/>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" s="5"/>
       <c r="B179" s="8"/>
       <c r="D179" s="12"/>
       <c r="E179" s="8"/>
-      <c r="F179" s="17"/>
+      <c r="F179" s="15"/>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" s="5"/>
       <c r="B180" s="8"/>
       <c r="D180" s="12"/>
       <c r="E180" s="8"/>
-      <c r="F180" s="17"/>
+      <c r="F180" s="15"/>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" s="5"/>
       <c r="B181" s="8"/>
       <c r="D181" s="12"/>
       <c r="E181" s="8"/>
-      <c r="F181" s="17"/>
+      <c r="F181" s="15"/>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" s="5"/>
       <c r="B182" s="8"/>
       <c r="D182" s="12"/>
       <c r="E182" s="8"/>
-      <c r="F182" s="17"/>
+      <c r="F182" s="15"/>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" s="5"/>
       <c r="B183" s="8"/>
       <c r="D183" s="12"/>
       <c r="E183" s="8"/>
-      <c r="F183" s="17"/>
+      <c r="F183" s="15"/>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" s="5"/>
       <c r="B184" s="8"/>
       <c r="D184" s="12"/>
       <c r="E184" s="8"/>
-      <c r="F184" s="17"/>
+      <c r="F184" s="15"/>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" s="5"/>
       <c r="B185" s="8"/>
       <c r="D185" s="12"/>
       <c r="E185" s="8"/>
-      <c r="F185" s="17"/>
+      <c r="F185" s="15"/>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" s="5"/>
       <c r="B186" s="8"/>
       <c r="D186" s="12"/>
       <c r="E186" s="8"/>
-      <c r="F186" s="17"/>
+      <c r="F186" s="15"/>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" s="5"/>
       <c r="B187" s="8"/>
       <c r="D187" s="12"/>
       <c r="E187" s="8"/>
-      <c r="F187" s="17"/>
+      <c r="F187" s="15"/>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" s="5"/>
       <c r="B188" s="8"/>
       <c r="D188" s="12"/>
       <c r="E188" s="8"/>
-      <c r="F188" s="17"/>
+      <c r="F188" s="15"/>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" s="5"/>
       <c r="B189" s="8"/>
       <c r="D189" s="12"/>
       <c r="E189" s="8"/>
-      <c r="F189" s="17"/>
+      <c r="F189" s="15"/>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" s="5"/>
       <c r="B190" s="8"/>
       <c r="D190" s="12"/>
       <c r="E190" s="8"/>
-      <c r="F190" s="17"/>
+      <c r="F190" s="15"/>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" s="5"/>
       <c r="B191" s="8"/>
       <c r="D191" s="12"/>
       <c r="E191" s="8"/>
-      <c r="F191" s="17"/>
+      <c r="F191" s="15"/>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" s="5"/>
       <c r="B192" s="8"/>
       <c r="D192" s="12"/>
       <c r="E192" s="8"/>
-      <c r="F192" s="17"/>
+      <c r="F192" s="15"/>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" s="5"/>
       <c r="B193" s="8"/>
       <c r="D193" s="12"/>
       <c r="E193" s="8"/>
-      <c r="F193" s="17"/>
+      <c r="F193" s="15"/>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" s="5"/>
       <c r="B194" s="8"/>
       <c r="D194" s="12"/>
       <c r="E194" s="8"/>
-      <c r="F194" s="17"/>
+      <c r="F194" s="15"/>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" s="5"/>
       <c r="B195" s="8"/>
       <c r="D195" s="12"/>
       <c r="E195" s="8"/>
-      <c r="F195" s="17"/>
+      <c r="F195" s="15"/>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" s="5"/>
       <c r="B196" s="8"/>
       <c r="D196" s="12"/>
       <c r="E196" s="8"/>
-      <c r="F196" s="17"/>
+      <c r="F196" s="15"/>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" s="5"/>
       <c r="B197" s="8"/>
       <c r="D197" s="12"/>
       <c r="E197" s="8"/>
-      <c r="F197" s="17"/>
+      <c r="F197" s="15"/>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" s="5"/>
       <c r="B198" s="8"/>
       <c r="D198" s="12"/>
       <c r="E198" s="8"/>
-      <c r="F198" s="17"/>
+      <c r="F198" s="15"/>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" s="5"/>
       <c r="B199" s="8"/>
       <c r="D199" s="12"/>
       <c r="E199" s="8"/>
-      <c r="F199" s="17"/>
+      <c r="F199" s="15"/>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" s="5"/>
       <c r="B200" s="8"/>
       <c r="D200" s="12"/>
       <c r="E200" s="8"/>
-      <c r="F200" s="17"/>
+      <c r="F200" s="15"/>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" s="5"/>
       <c r="B201" s="8"/>
       <c r="D201" s="12"/>
       <c r="E201" s="8"/>
-      <c r="F201" s="17"/>
+      <c r="F201" s="15"/>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" s="5"/>
       <c r="B202" s="9"/>
       <c r="D202" s="12"/>
       <c r="E202" s="8"/>
-      <c r="F202" s="17"/>
+      <c r="F202" s="15"/>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" s="5"/>
       <c r="B203" s="11"/>
       <c r="D203" s="12"/>
       <c r="E203" s="8"/>
-      <c r="F203" s="17"/>
+      <c r="F203" s="15"/>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" s="5"/>
       <c r="B204" s="9"/>
       <c r="D204" s="12"/>
       <c r="E204" s="8"/>
-      <c r="F204" s="17"/>
+      <c r="F204" s="15"/>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" s="5"/>
       <c r="B205" s="9"/>
       <c r="D205" s="12"/>
       <c r="E205" s="8"/>
-      <c r="F205" s="17"/>
+      <c r="F205" s="15"/>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" s="5"/>
       <c r="B206" s="9"/>
       <c r="D206" s="12"/>
       <c r="E206" s="8"/>
-      <c r="F206" s="17"/>
+      <c r="F206" s="15"/>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" s="5"/>
       <c r="B207" s="9"/>
       <c r="D207" s="12"/>
       <c r="E207" s="8"/>
-      <c r="F207" s="17"/>
+      <c r="F207" s="15"/>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" s="5"/>
       <c r="B208" s="9"/>
       <c r="D208" s="12"/>
       <c r="E208" s="8"/>
-      <c r="F208" s="17"/>
+      <c r="F208" s="15"/>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209" s="5"/>
       <c r="B209" s="9"/>
       <c r="D209" s="12"/>
       <c r="E209" s="8"/>
-      <c r="F209" s="17"/>
+      <c r="F209" s="15"/>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210" s="5"/>
       <c r="B210" s="9"/>
       <c r="D210" s="12"/>
       <c r="E210" s="8"/>
-      <c r="F210" s="17"/>
+      <c r="F210" s="15"/>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" s="5"/>
       <c r="B211" s="9"/>
       <c r="D211" s="12"/>
       <c r="E211" s="8"/>
-      <c r="F211" s="17"/>
+      <c r="F211" s="15"/>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212" s="5"/>
       <c r="B212" s="9"/>
       <c r="D212" s="12"/>
       <c r="E212" s="8"/>
-      <c r="F212" s="17"/>
+      <c r="F212" s="15"/>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A213" s="5"/>
       <c r="B213" s="9"/>
       <c r="D213" s="12"/>
       <c r="E213" s="8"/>
-      <c r="F213" s="17"/>
+      <c r="F213" s="15"/>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214" s="5"/>
       <c r="B214" s="9"/>
       <c r="D214" s="12"/>
       <c r="E214" s="8"/>
-      <c r="F214" s="17"/>
+      <c r="F214" s="15"/>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A215" s="5"/>
       <c r="B215" s="9"/>
       <c r="D215" s="12"/>
       <c r="E215" s="8"/>
-      <c r="F215" s="17"/>
+      <c r="F215" s="15"/>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A216" s="5"/>
       <c r="B216" s="9"/>
       <c r="D216" s="12"/>
       <c r="E216" s="8"/>
-      <c r="F216" s="17"/>
+      <c r="F216" s="15"/>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217" s="5"/>
       <c r="B217" s="9"/>
       <c r="D217" s="12"/>
       <c r="E217" s="8"/>
-      <c r="F217" s="17"/>
+      <c r="F217" s="15"/>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218" s="5"/>
       <c r="B218" s="9"/>
       <c r="D218" s="12"/>
       <c r="E218" s="8"/>
-      <c r="F218" s="17"/>
+      <c r="F218" s="15"/>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A219" s="5"/>
       <c r="B219" s="9"/>
       <c r="D219" s="12"/>
       <c r="E219" s="8"/>
-      <c r="F219" s="17"/>
+      <c r="F219" s="15"/>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A220" s="5"/>
       <c r="B220" s="9"/>
       <c r="D220" s="12"/>
       <c r="E220" s="8"/>
-      <c r="F220" s="17"/>
+      <c r="F220" s="15"/>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A221" s="5"/>
       <c r="B221" s="9"/>
       <c r="D221" s="12"/>
       <c r="E221" s="8"/>
-      <c r="F221" s="17"/>
+      <c r="F221" s="15"/>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A222" s="5"/>
       <c r="B222" s="9"/>
       <c r="D222" s="12"/>
       <c r="E222" s="8"/>
-      <c r="F222" s="17"/>
+      <c r="F222" s="15"/>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A223" s="5"/>
       <c r="B223" s="9"/>
       <c r="D223" s="12"/>
       <c r="E223" s="8"/>
-      <c r="F223" s="17"/>
+      <c r="F223" s="15"/>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A224" s="5"/>
       <c r="B224" s="9"/>
       <c r="D224" s="12"/>
       <c r="E224" s="8"/>
-      <c r="F224" s="17"/>
+      <c r="F224" s="15"/>
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A225" s="5"/>
       <c r="B225" s="9"/>
       <c r="D225" s="12"/>
       <c r="E225" s="8"/>
-      <c r="F225" s="17"/>
+      <c r="F225" s="15"/>
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A226" s="5"/>
       <c r="B226" s="9"/>
       <c r="D226" s="12"/>
       <c r="E226" s="8"/>
-      <c r="F226" s="17"/>
+      <c r="F226" s="15"/>
     </row>
     <row r="227" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A227" s="5"/>
       <c r="B227" s="9"/>
       <c r="D227" s="12"/>
       <c r="E227" s="8"/>
-      <c r="F227" s="17"/>
+      <c r="F227" s="15"/>
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A228" s="5"/>
       <c r="B228" s="9"/>
       <c r="D228" s="12"/>
       <c r="E228" s="8"/>
-      <c r="F228" s="17"/>
+      <c r="F228" s="15"/>
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A229" s="5"/>
       <c r="B229" s="9"/>
       <c r="D229" s="12"/>
       <c r="E229" s="8"/>
-      <c r="F229" s="17"/>
+      <c r="F229" s="15"/>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A230" s="5"/>
       <c r="B230" s="9"/>
       <c r="D230" s="12"/>
       <c r="E230" s="8"/>
-      <c r="F230" s="17"/>
+      <c r="F230" s="15"/>
     </row>
     <row r="231" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A231" s="5"/>
       <c r="B231" s="9"/>
       <c r="D231" s="12"/>
       <c r="E231" s="8"/>
-      <c r="F231" s="17"/>
+      <c r="F231" s="15"/>
     </row>
     <row r="232" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A232" s="5"/>
       <c r="B232" s="9"/>
       <c r="D232" s="12"/>
       <c r="E232" s="8"/>
-      <c r="F232" s="17"/>
+      <c r="F232" s="15"/>
     </row>
     <row r="233" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A233" s="5"/>
       <c r="B233" s="9"/>
       <c r="D233" s="12"/>
       <c r="E233" s="8"/>
-      <c r="F233" s="17"/>
+      <c r="F233" s="15"/>
     </row>
     <row r="234" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A234" s="5"/>
       <c r="B234" s="9"/>
       <c r="D234" s="12"/>
       <c r="E234" s="8"/>
-      <c r="F234" s="17"/>
+      <c r="F234" s="15"/>
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A235" s="5"/>
       <c r="B235" s="9"/>
       <c r="D235" s="12"/>
       <c r="E235" s="8"/>
-      <c r="F235" s="17"/>
+      <c r="F235" s="15"/>
     </row>
     <row r="236" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A236" s="5"/>
       <c r="B236" s="9"/>
       <c r="D236" s="12"/>
       <c r="E236" s="8"/>
-      <c r="F236" s="17"/>
+      <c r="F236" s="15"/>
     </row>
     <row r="237" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A237" s="5"/>
       <c r="B237" s="9"/>
       <c r="D237" s="12"/>
       <c r="E237" s="8"/>
-      <c r="F237" s="17"/>
+      <c r="F237" s="15"/>
     </row>
     <row r="238" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A238" s="5"/>
       <c r="B238" s="9"/>
       <c r="D238" s="12"/>
       <c r="E238" s="8"/>
-      <c r="F238" s="17"/>
+      <c r="F238" s="15"/>
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A239" s="5"/>
       <c r="B239" s="9"/>
       <c r="D239" s="12"/>
       <c r="E239" s="8"/>
-      <c r="F239" s="17"/>
+      <c r="F239" s="15"/>
     </row>
     <row r="240" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A240" s="5"/>
       <c r="B240" s="9"/>
       <c r="D240" s="12"/>
       <c r="E240" s="8"/>
-      <c r="F240" s="17"/>
+      <c r="F240" s="15"/>
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A241" s="5"/>
       <c r="B241" s="9"/>
       <c r="D241" s="12"/>
       <c r="E241" s="8"/>
-      <c r="F241" s="17"/>
+      <c r="F241" s="15"/>
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A242" s="5"/>
       <c r="B242" s="9"/>
       <c r="D242" s="12"/>
       <c r="E242" s="8"/>
-      <c r="F242" s="17"/>
+      <c r="F242" s="15"/>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A243" s="5"/>
       <c r="B243" s="9"/>
       <c r="D243" s="12"/>
       <c r="E243" s="8"/>
-      <c r="F243" s="17"/>
+      <c r="F243" s="15"/>
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A244" s="5"/>
       <c r="B244" s="9"/>
       <c r="D244" s="12"/>
       <c r="E244" s="8"/>
-      <c r="F244" s="17"/>
+      <c r="F244" s="15"/>
     </row>
     <row r="245" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A245" s="5"/>
       <c r="B245" s="9"/>
       <c r="D245" s="12"/>
       <c r="E245" s="8"/>
-      <c r="F245" s="17"/>
+      <c r="F245" s="15"/>
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A246" s="5"/>
       <c r="B246" s="9"/>
       <c r="D246" s="12"/>
       <c r="E246" s="8"/>
-      <c r="F246" s="17"/>
+      <c r="F246" s="15"/>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A247" s="5"/>
       <c r="B247" s="9"/>
       <c r="D247" s="12"/>
       <c r="E247" s="8"/>
-      <c r="F247" s="17"/>
+      <c r="F247" s="15"/>
     </row>
     <row r="248" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A248" s="5"/>
       <c r="B248" s="9"/>
       <c r="D248" s="12"/>
       <c r="E248" s="8"/>
-      <c r="F248" s="17"/>
+      <c r="F248" s="15"/>
     </row>
     <row r="249" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A249" s="5"/>
       <c r="B249" s="9"/>
       <c r="D249" s="12"/>
       <c r="E249" s="8"/>
-      <c r="F249" s="17"/>
+      <c r="F249" s="15"/>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A250" s="5"/>
       <c r="B250" s="9"/>
       <c r="D250" s="12"/>
       <c r="E250" s="8"/>
-      <c r="F250" s="17"/>
+      <c r="F250" s="15"/>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A251" s="5"/>
       <c r="B251" s="9"/>
       <c r="D251" s="12"/>
       <c r="E251" s="8"/>
-      <c r="F251" s="17"/>
+      <c r="F251" s="15"/>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A252" s="5"/>
       <c r="B252" s="9"/>
       <c r="D252" s="12"/>
       <c r="E252" s="8"/>
-      <c r="F252" s="17"/>
+      <c r="F252" s="15"/>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A253" s="5"/>
       <c r="B253" s="9"/>
       <c r="D253" s="12"/>
       <c r="E253" s="8"/>
-      <c r="F253" s="17"/>
+      <c r="F253" s="15"/>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A254" s="5"/>
       <c r="B254" s="9"/>
       <c r="D254" s="12"/>
       <c r="E254" s="8"/>
-      <c r="F254" s="17"/>
+      <c r="F254" s="15"/>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A255" s="5"/>
       <c r="B255" s="9"/>
       <c r="D255" s="12"/>
       <c r="E255" s="8"/>
-      <c r="F255" s="17"/>
+      <c r="F255" s="15"/>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A256" s="5"/>
       <c r="B256" s="9"/>
       <c r="D256" s="12"/>
       <c r="E256" s="8"/>
-      <c r="F256" s="17"/>
+      <c r="F256" s="15"/>
     </row>
     <row r="257" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A257" s="5"/>
       <c r="B257" s="9"/>
       <c r="D257" s="12"/>
       <c r="E257" s="8"/>
-      <c r="F257" s="17"/>
+      <c r="F257" s="15"/>
     </row>
     <row r="258" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A258" s="5"/>
       <c r="B258" s="9"/>
       <c r="D258" s="12"/>
       <c r="E258" s="8"/>
-      <c r="F258" s="17"/>
+      <c r="F258" s="15"/>
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A259" s="5"/>
       <c r="B259" s="9"/>
       <c r="D259" s="12"/>
       <c r="E259" s="8"/>
-      <c r="F259" s="17"/>
+      <c r="F259" s="15"/>
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A260" s="5"/>
       <c r="B260" s="9"/>
       <c r="D260" s="12"/>
       <c r="E260" s="8"/>
-      <c r="F260" s="17"/>
+      <c r="F260" s="15"/>
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A261" s="5"/>
       <c r="B261" s="9"/>
       <c r="D261" s="12"/>
       <c r="E261" s="8"/>
-      <c r="F261" s="17"/>
+      <c r="F261" s="15"/>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A262" s="5"/>
       <c r="B262" s="9"/>
       <c r="D262" s="12"/>
       <c r="E262" s="8"/>
-      <c r="F262" s="17"/>
+      <c r="F262" s="15"/>
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A263" s="5"/>
       <c r="B263" s="9"/>
       <c r="D263" s="12"/>
       <c r="E263" s="8"/>
-      <c r="F263" s="17"/>
+      <c r="F263" s="15"/>
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A264" s="5"/>
       <c r="B264" s="9"/>
       <c r="D264" s="12"/>
       <c r="E264" s="8"/>
-      <c r="F264" s="17"/>
+      <c r="F264" s="15"/>
     </row>
     <row r="265" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A265" s="5"/>
       <c r="B265" s="9"/>
       <c r="D265" s="12"/>
       <c r="E265" s="8"/>
-      <c r="F265" s="17"/>
+      <c r="F265" s="15"/>
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A266" s="5"/>
       <c r="B266" s="9"/>
       <c r="D266" s="12"/>
       <c r="E266" s="8"/>
-      <c r="F266" s="17"/>
+      <c r="F266" s="15"/>
     </row>
     <row r="267" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A267" s="5"/>
       <c r="B267" s="9"/>
       <c r="D267" s="12"/>
       <c r="E267" s="8"/>
-      <c r="F267" s="17"/>
+      <c r="F267" s="15"/>
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A268" s="5"/>
       <c r="B268" s="9"/>
       <c r="D268" s="12"/>
       <c r="E268" s="8"/>
-      <c r="F268" s="17"/>
+      <c r="F268" s="15"/>
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A269" s="5"/>
       <c r="B269" s="9"/>
       <c r="D269" s="12"/>
       <c r="E269" s="8"/>
-      <c r="F269" s="17"/>
+      <c r="F269" s="15"/>
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A270" s="5"/>
       <c r="B270" s="9"/>
       <c r="D270" s="12"/>
       <c r="E270" s="8"/>
-      <c r="F270" s="17"/>
+      <c r="F270" s="15"/>
     </row>
     <row r="271" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A271" s="5"/>
       <c r="B271" s="9"/>
       <c r="D271" s="12"/>
       <c r="E271" s="8"/>
-      <c r="F271" s="17"/>
+      <c r="F271" s="15"/>
     </row>
     <row r="272" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A272" s="5"/>
       <c r="B272" s="9"/>
       <c r="D272" s="12"/>
       <c r="E272" s="8"/>
-      <c r="F272" s="17"/>
+      <c r="F272" s="15"/>
     </row>
     <row r="273" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A273" s="5"/>
       <c r="B273" s="9"/>
       <c r="D273" s="12"/>
       <c r="E273" s="8"/>
-      <c r="F273" s="17"/>
+      <c r="F273" s="15"/>
     </row>
     <row r="274" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A274" s="5"/>
       <c r="B274" s="9"/>
       <c r="D274" s="12"/>
       <c r="E274" s="8"/>
-      <c r="F274" s="17"/>
+      <c r="F274" s="15"/>
     </row>
     <row r="275" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A275" s="5"/>
       <c r="B275" s="9"/>
       <c r="D275" s="12"/>
       <c r="E275" s="8"/>
-      <c r="F275" s="17"/>
+      <c r="F275" s="15"/>
     </row>
     <row r="276" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A276" s="5"/>
       <c r="B276" s="9"/>
       <c r="D276" s="12"/>
       <c r="E276" s="8"/>
-      <c r="F276" s="17"/>
+      <c r="F276" s="15"/>
     </row>
     <row r="277" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A277" s="5"/>
       <c r="B277" s="9"/>
       <c r="D277" s="12"/>
       <c r="E277" s="8"/>
-      <c r="F277" s="17"/>
+      <c r="F277" s="15"/>
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A278" s="5"/>
       <c r="B278" s="9"/>
       <c r="D278" s="12"/>
       <c r="E278" s="8"/>
-      <c r="F278" s="17"/>
+      <c r="F278" s="15"/>
     </row>
     <row r="279" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A279" s="5"/>
       <c r="B279" s="8"/>
       <c r="D279" s="12"/>
       <c r="E279" s="8"/>
-      <c r="F279" s="17"/>
+      <c r="F279" s="15"/>
     </row>
     <row r="280" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A280" s="5"/>
       <c r="B280" s="8"/>
       <c r="D280" s="12"/>
       <c r="E280" s="8"/>
-      <c r="F280" s="17"/>
+      <c r="F280" s="15"/>
     </row>
     <row r="281" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A281" s="5"/>
       <c r="B281" s="8"/>
       <c r="D281" s="12"/>
       <c r="E281" s="8"/>
-      <c r="F281" s="17"/>
+      <c r="F281" s="15"/>
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A282" s="5"/>
       <c r="B282" s="8"/>
       <c r="D282" s="12"/>
       <c r="E282" s="8"/>
-      <c r="F282" s="17"/>
+      <c r="F282" s="15"/>
     </row>
     <row r="283" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A283" s="5"/>
       <c r="B283" s="8"/>
       <c r="D283" s="12"/>
       <c r="E283" s="8"/>
-      <c r="F283" s="17"/>
+      <c r="F283" s="15"/>
     </row>
     <row r="284" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A284" s="5"/>

</xml_diff>